<commit_message>
feat: added illustration in the hero section and made the code more modular
</commit_message>
<xml_diff>
--- a/try_ExamDuty.xlsx
+++ b/try_ExamDuty.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="42">
   <si>
     <t>Faculty</t>
   </si>
@@ -19,121 +19,124 @@
     <t>Staff</t>
   </si>
   <si>
-    <t>Dr. Sharma</t>
-  </si>
-  <si>
-    <t>Mr. Verma</t>
-  </si>
-  <si>
-    <t>Dr. Malviya</t>
-  </si>
-  <si>
-    <t>Mr. Naidu</t>
-  </si>
-  <si>
-    <t>Dr. Mishra</t>
-  </si>
-  <si>
-    <t>Mr. Rao</t>
-  </si>
-  <si>
-    <t>Dr. Mahto</t>
-  </si>
-  <si>
-    <t>Mr. Singh</t>
-  </si>
-  <si>
-    <t>Dr. Yadav</t>
-  </si>
-  <si>
-    <t>Mr. Kumar</t>
-  </si>
-  <si>
-    <t>Dr. Panda</t>
-  </si>
-  <si>
-    <t>Mr. Das</t>
-  </si>
-  <si>
-    <t>Dr. Choudhary</t>
-  </si>
-  <si>
-    <t>Mr. Joshi</t>
-  </si>
-  <si>
-    <t>Dr. Banerjee</t>
-  </si>
-  <si>
-    <t>Mr. Gupta</t>
-  </si>
-  <si>
-    <t>Dr. Malhotra</t>
-  </si>
-  <si>
-    <t>Mr. Patel</t>
-  </si>
-  <si>
-    <t>Dr. Saxena</t>
-  </si>
-  <si>
-    <t>Mr. Mishra</t>
-  </si>
-  <si>
-    <t>Dr. Kulkarni</t>
-  </si>
-  <si>
-    <t>Dr. Pillai</t>
-  </si>
-  <si>
-    <t>Dr. Deshmukh</t>
-  </si>
-  <si>
-    <t>Dr. Bhatia</t>
-  </si>
-  <si>
-    <t>Dr. Kapoor</t>
-  </si>
-  <si>
-    <t>Dr. Srivastava</t>
-  </si>
-  <si>
-    <t>Dr. Trivedi</t>
-  </si>
-  <si>
-    <t>Dr. Bhattacharya</t>
-  </si>
-  <si>
-    <t>Dr. Pandey</t>
-  </si>
-  <si>
-    <t>Dr. Thakur</t>
-  </si>
-  <si>
-    <t>Dr. Goswami</t>
-  </si>
-  <si>
-    <t>Dr. Arora</t>
-  </si>
-  <si>
-    <t>Dr. Menon</t>
-  </si>
-  <si>
-    <t>Dr. Khanna</t>
-  </si>
-  <si>
-    <t>Dr. Sinha</t>
-  </si>
-  <si>
-    <t>Dr. Shetty</t>
-  </si>
-  <si>
-    <t>Dr. Dubey</t>
-  </si>
-  <si>
-    <t>Dr. Purohit</t>
-  </si>
-  <si>
-    <t>Dr. Jain</t>
+    <t>Faculty 1</t>
+  </si>
+  <si>
+    <t>Staff 1</t>
+  </si>
+  <si>
+    <t>Faculty 2</t>
+  </si>
+  <si>
+    <t>Staff 2</t>
+  </si>
+  <si>
+    <t>Faculty 3</t>
+  </si>
+  <si>
+    <t>Staff 3</t>
+  </si>
+  <si>
+    <t>Faculty 4</t>
+  </si>
+  <si>
+    <t>Staff 4</t>
+  </si>
+  <si>
+    <t>Faculty 5</t>
+  </si>
+  <si>
+    <t>Staff 5</t>
+  </si>
+  <si>
+    <t>Faculty 6</t>
+  </si>
+  <si>
+    <t>Staff 6</t>
+  </si>
+  <si>
+    <t>Faculty 7</t>
+  </si>
+  <si>
+    <t>Staff 7</t>
+  </si>
+  <si>
+    <t>Faculty 8</t>
+  </si>
+  <si>
+    <t>Staff 8</t>
+  </si>
+  <si>
+    <t>Faculty 9</t>
+  </si>
+  <si>
+    <t>Staff 9</t>
+  </si>
+  <si>
+    <t>Faculty 10</t>
+  </si>
+  <si>
+    <t>Staff 10</t>
+  </si>
+  <si>
+    <t>Faculty 11</t>
+  </si>
+  <si>
+    <t>Faculty 12</t>
+  </si>
+  <si>
+    <t>Faculty 13</t>
+  </si>
+  <si>
+    <t>Faculty 14</t>
+  </si>
+  <si>
+    <t>Faculty 15</t>
+  </si>
+  <si>
+    <t>Faculty 16</t>
+  </si>
+  <si>
+    <t>Faculty 17</t>
+  </si>
+  <si>
+    <t>Faculty 18</t>
+  </si>
+  <si>
+    <t>Faculty 19</t>
+  </si>
+  <si>
+    <t>Faculty 20</t>
+  </si>
+  <si>
+    <t>Faculty 21</t>
+  </si>
+  <si>
+    <t>Faculty 22</t>
+  </si>
+  <si>
+    <t>Faculty 23</t>
+  </si>
+  <si>
+    <t>Faculty 24</t>
+  </si>
+  <si>
+    <t>Faculty 25</t>
+  </si>
+  <si>
+    <t>Faculty 26</t>
+  </si>
+  <si>
+    <t>Faculty 27</t>
+  </si>
+  <si>
+    <t>Faculty 28</t>
+  </si>
+  <si>
+    <t>Faculty 29</t>
+  </si>
+  <si>
+    <t>Faculty 30</t>
   </si>
 </sst>
 </file>
@@ -143,9 +146,9 @@
   <numFmts count="1">
     <numFmt numFmtId="0" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="3">
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color indexed="8"/>
       <name val="Calibri"/>
     </font>
@@ -159,24 +162,19 @@
       <color indexed="8"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Times Roman"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Times Roman"/>
-    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="9"/>
+        <bgColor auto="1"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -189,16 +187,16 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </left>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
@@ -208,21 +206,18 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="3" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="4" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -241,6 +236,7 @@
       <rgbColor rgb="ffff00ff"/>
       <rgbColor rgb="ff00ffff"/>
       <rgbColor rgb="ff000000"/>
+      <rgbColor rgb="ffffffff"/>
       <rgbColor rgb="ffaaaaaa"/>
     </indexedColors>
   </colors>
@@ -264,22 +260,22 @@
         <a:srgbClr val="535353"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
         <a:srgbClr val="0000FF"/>
@@ -373,13 +369,31 @@
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -440,17 +454,23 @@
         <a:solidFill>
           <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
-        <a:ln w="12700" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:round/>
         </a:ln>
-        <a:effectLst/>
+        <a:effectLst>
+          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
+            <a:srgbClr val="000000">
+              <a:alpha val="35000"/>
+            </a:srgbClr>
+          </a:outerShdw>
+        </a:effectLst>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -477,10 +497,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -719,14 +739,20 @@
     <a:lnDef>
       <a:spPr>
         <a:noFill/>
-        <a:ln w="12700" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:round/>
         </a:ln>
-        <a:effectLst/>
+        <a:effectLst>
+          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
+            <a:srgbClr val="000000">
+              <a:alpha val="35000"/>
+            </a:srgbClr>
+          </a:outerShdw>
+        </a:effectLst>
         <a:sp3d/>
       </a:spPr>
       <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
@@ -1001,7 +1027,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1028,10 +1054,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -1273,218 +1299,319 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="14.4" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E31"/>
+  <sheetFormatPr defaultColWidth="8" defaultRowHeight="12.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="14.6719" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.85156" style="1" customWidth="1"/>
+    <col min="1" max="5" width="8" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="8" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17" customHeight="1">
+    <row r="1" ht="15.35" customHeight="1">
       <c r="A1" t="s" s="2">
         <v>0</v>
       </c>
       <c r="B1" t="s" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" ht="17" customHeight="1">
-      <c r="A2" t="s" s="3">
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+    </row>
+    <row r="2" ht="15.35" customHeight="1">
+      <c r="A2" t="s" s="2">
         <v>2</v>
       </c>
-      <c r="B2" t="s" s="3">
+      <c r="B2" t="s" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" ht="17" customHeight="1">
-      <c r="A3" t="s" s="3">
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+    </row>
+    <row r="3" ht="15.35" customHeight="1">
+      <c r="A3" t="s" s="2">
         <v>4</v>
       </c>
-      <c r="B3" t="s" s="3">
+      <c r="B3" t="s" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" ht="17" customHeight="1">
-      <c r="A4" t="s" s="3">
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+    </row>
+    <row r="4" ht="15.35" customHeight="1">
+      <c r="A4" t="s" s="2">
         <v>6</v>
       </c>
-      <c r="B4" t="s" s="3">
+      <c r="B4" t="s" s="2">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" ht="17" customHeight="1">
-      <c r="A5" t="s" s="3">
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+    </row>
+    <row r="5" ht="15.35" customHeight="1">
+      <c r="A5" t="s" s="2">
         <v>8</v>
       </c>
-      <c r="B5" t="s" s="3">
+      <c r="B5" t="s" s="2">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" ht="17" customHeight="1">
-      <c r="A6" t="s" s="3">
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+    </row>
+    <row r="6" ht="15.35" customHeight="1">
+      <c r="A6" t="s" s="2">
         <v>10</v>
       </c>
-      <c r="B6" t="s" s="3">
+      <c r="B6" t="s" s="2">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" ht="17" customHeight="1">
-      <c r="A7" t="s" s="3">
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+    </row>
+    <row r="7" ht="15.35" customHeight="1">
+      <c r="A7" t="s" s="2">
         <v>12</v>
       </c>
-      <c r="B7" t="s" s="3">
+      <c r="B7" t="s" s="2">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" t="s" s="3">
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+    </row>
+    <row r="8" ht="15.35" customHeight="1">
+      <c r="A8" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="B8" t="s" s="3">
+      <c r="B8" t="s" s="2">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" ht="17" customHeight="1">
-      <c r="A9" t="s" s="3">
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+    </row>
+    <row r="9" ht="15.35" customHeight="1">
+      <c r="A9" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="B9" t="s" s="3">
+      <c r="B9" t="s" s="2">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" ht="17" customHeight="1">
-      <c r="A10" t="s" s="3">
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+    </row>
+    <row r="10" ht="15.35" customHeight="1">
+      <c r="A10" t="s" s="2">
         <v>18</v>
       </c>
-      <c r="B10" t="s" s="3">
+      <c r="B10" t="s" s="2">
         <v>19</v>
       </c>
-    </row>
-    <row r="11" ht="17" customHeight="1">
-      <c r="A11" t="s" s="3">
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+    </row>
+    <row r="11" ht="15.35" customHeight="1">
+      <c r="A11" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="B11" t="s" s="3">
+      <c r="B11" t="s" s="2">
         <v>21</v>
       </c>
-    </row>
-    <row r="12" ht="17" customHeight="1">
-      <c r="A12" t="s" s="3">
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+    </row>
+    <row r="12" ht="15.35" customHeight="1">
+      <c r="A12" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="B12" s="4"/>
-    </row>
-    <row r="13" ht="17" customHeight="1">
-      <c r="A13" t="s" s="3">
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+    </row>
+    <row r="13" ht="15.35" customHeight="1">
+      <c r="A13" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="B13" s="4"/>
-    </row>
-    <row r="14" ht="17" customHeight="1">
-      <c r="A14" t="s" s="3">
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+    </row>
+    <row r="14" ht="15.35" customHeight="1">
+      <c r="A14" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="B14" s="4"/>
-    </row>
-    <row r="15" ht="17" customHeight="1">
-      <c r="A15" t="s" s="3">
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+    </row>
+    <row r="15" ht="15.35" customHeight="1">
+      <c r="A15" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="B15" s="4"/>
-    </row>
-    <row r="16" ht="17" customHeight="1">
-      <c r="A16" t="s" s="3">
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+    </row>
+    <row r="16" ht="15.35" customHeight="1">
+      <c r="A16" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="B16" s="4"/>
-    </row>
-    <row r="17" ht="17" customHeight="1">
-      <c r="A17" t="s" s="3">
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+    </row>
+    <row r="17" ht="15.35" customHeight="1">
+      <c r="A17" t="s" s="2">
         <v>27</v>
       </c>
-      <c r="B17" s="4"/>
-    </row>
-    <row r="18" ht="17" customHeight="1">
-      <c r="A18" t="s" s="3">
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" ht="15.35" customHeight="1">
+      <c r="A18" t="s" s="2">
         <v>28</v>
       </c>
-      <c r="B18" s="4"/>
-    </row>
-    <row r="19" ht="17" customHeight="1">
-      <c r="A19" t="s" s="3">
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+    </row>
+    <row r="19" ht="15.35" customHeight="1">
+      <c r="A19" t="s" s="2">
         <v>29</v>
       </c>
-      <c r="B19" s="4"/>
-    </row>
-    <row r="20" ht="17" customHeight="1">
-      <c r="A20" t="s" s="3">
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+    </row>
+    <row r="20" ht="15.35" customHeight="1">
+      <c r="A20" t="s" s="2">
         <v>30</v>
       </c>
-      <c r="B20" s="4"/>
-    </row>
-    <row r="21" ht="17" customHeight="1">
-      <c r="A21" t="s" s="3">
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+    </row>
+    <row r="21" ht="15.35" customHeight="1">
+      <c r="A21" t="s" s="2">
         <v>31</v>
       </c>
-      <c r="B21" s="4"/>
-    </row>
-    <row r="22" ht="17" customHeight="1">
-      <c r="A22" t="s" s="3">
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+    </row>
+    <row r="22" ht="15.35" customHeight="1">
+      <c r="A22" t="s" s="2">
         <v>32</v>
       </c>
-      <c r="B22" s="4"/>
-    </row>
-    <row r="23" ht="17" customHeight="1">
-      <c r="A23" t="s" s="3">
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+    </row>
+    <row r="23" ht="15.35" customHeight="1">
+      <c r="A23" t="s" s="2">
         <v>33</v>
       </c>
-      <c r="B23" s="4"/>
-    </row>
-    <row r="24" ht="17" customHeight="1">
-      <c r="A24" t="s" s="3">
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+    </row>
+    <row r="24" ht="15.35" customHeight="1">
+      <c r="A24" t="s" s="2">
         <v>34</v>
       </c>
-      <c r="B24" s="4"/>
-    </row>
-    <row r="25" ht="17" customHeight="1">
-      <c r="A25" t="s" s="3">
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+    </row>
+    <row r="25" ht="15.35" customHeight="1">
+      <c r="A25" t="s" s="2">
         <v>35</v>
       </c>
-      <c r="B25" s="4"/>
-    </row>
-    <row r="26" ht="17" customHeight="1">
-      <c r="A26" t="s" s="3">
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+    </row>
+    <row r="26" ht="15.35" customHeight="1">
+      <c r="A26" t="s" s="2">
         <v>36</v>
       </c>
-      <c r="B26" s="4"/>
-    </row>
-    <row r="27" ht="17" customHeight="1">
-      <c r="A27" t="s" s="3">
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+    </row>
+    <row r="27" ht="15.35" customHeight="1">
+      <c r="A27" t="s" s="2">
         <v>37</v>
       </c>
-      <c r="B27" s="4"/>
-    </row>
-    <row r="28" ht="17" customHeight="1">
-      <c r="A28" t="s" s="3">
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+    </row>
+    <row r="28" ht="15.35" customHeight="1">
+      <c r="A28" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="B28" s="4"/>
-    </row>
-    <row r="29" ht="17" customHeight="1">
-      <c r="A29" t="s" s="3">
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+    </row>
+    <row r="29" ht="15.35" customHeight="1">
+      <c r="A29" t="s" s="2">
         <v>39</v>
       </c>
-      <c r="B29" s="4"/>
-    </row>
-    <row r="30" ht="17" customHeight="1">
-      <c r="A30" t="s" s="3">
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+    </row>
+    <row r="30" ht="15.35" customHeight="1">
+      <c r="A30" t="s" s="2">
         <v>40</v>
       </c>
-      <c r="B30" s="4"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+    </row>
+    <row r="31" ht="15.35" customHeight="1">
+      <c r="A31" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>

</xml_diff>